<commit_message>
Update the figures and include new ones
</commit_message>
<xml_diff>
--- a/outputs/dataframes/health_counts.xlsx
+++ b/outputs/dataframes/health_counts.xlsx
@@ -107750,13 +107750,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D13B18A5-B5A4-46C1-9723-5B1A77F2670A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7794EBCA-0C36-49D4-A180-1F53AECCC855}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A1221F4-3A90-4A96-A9B1-B3C4630F1A46}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE28097A-25CE-4F34-BAF8-0D22A97BF507}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA07B6A0-A0C7-48A8-8D73-A08FBF80754E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C07BDE9-0CB3-4FF7-B573-757BCE15BDA7}"/>
 </file>
</xml_diff>

<commit_message>
Update the health counts data
</commit_message>
<xml_diff>
--- a/outputs/dataframes/health_counts.xlsx
+++ b/outputs/dataframes/health_counts.xlsx
@@ -8421,10 +8421,10 @@
         </is>
       </c>
       <c r="AD30" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="AE30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF30" t="n">
         <v>0</v>
@@ -8433,7 +8433,7 @@
         <v>1</v>
       </c>
       <c r="AH30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI30" t="n">
         <v>1</v>
@@ -8481,7 +8481,7 @@
         <v>0</v>
       </c>
       <c r="AX30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
@@ -8565,10 +8565,10 @@
         </is>
       </c>
       <c r="AD31" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="AE31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF31" t="n">
         <v>0</v>
@@ -8577,7 +8577,7 @@
         <v>1</v>
       </c>
       <c r="AH31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI31" t="n">
         <v>1</v>
@@ -8625,7 +8625,7 @@
         <v>0</v>
       </c>
       <c r="AX31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
@@ -8709,10 +8709,10 @@
         </is>
       </c>
       <c r="AD32" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="AE32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF32" t="n">
         <v>0</v>
@@ -8721,7 +8721,7 @@
         <v>1</v>
       </c>
       <c r="AH32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI32" t="n">
         <v>1</v>
@@ -8769,7 +8769,7 @@
         <v>0</v>
       </c>
       <c r="AX32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
@@ -8853,67 +8853,67 @@
         </is>
       </c>
       <c r="AD33" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="AE33" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX33" t="n">
         <v>4</v>
-      </c>
-      <c r="AF33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG33" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN33" t="n">
-        <v>2</v>
-      </c>
-      <c r="AO33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AU33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AW33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX33" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="34">
@@ -8997,10 +8997,10 @@
         </is>
       </c>
       <c r="AD34" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="AE34" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AF34" t="n">
         <v>0</v>
@@ -9009,7 +9009,7 @@
         <v>4</v>
       </c>
       <c r="AH34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI34" t="n">
         <v>2</v>
@@ -9057,7 +9057,7 @@
         <v>0</v>
       </c>
       <c r="AX34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
@@ -9141,10 +9141,10 @@
         </is>
       </c>
       <c r="AD35" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="AE35" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AF35" t="n">
         <v>0</v>
@@ -9153,7 +9153,7 @@
         <v>4</v>
       </c>
       <c r="AH35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI35" t="n">
         <v>2</v>
@@ -9201,7 +9201,7 @@
         <v>0</v>
       </c>
       <c r="AX35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36">
@@ -9285,10 +9285,10 @@
         </is>
       </c>
       <c r="AD36" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="AE36" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AF36" t="n">
         <v>0</v>
@@ -9297,7 +9297,7 @@
         <v>4</v>
       </c>
       <c r="AH36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI36" t="n">
         <v>2</v>
@@ -9345,7 +9345,7 @@
         <v>0</v>
       </c>
       <c r="AX36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="37">
@@ -9429,43 +9429,43 @@
         </is>
       </c>
       <c r="AD37" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="AE37" t="n">
+        <v>9</v>
+      </c>
+      <c r="AF37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG37" t="n">
         <v>6</v>
       </c>
-      <c r="AF37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG37" t="n">
+      <c r="AH37" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI37" t="n">
+        <v>3</v>
+      </c>
+      <c r="AJ37" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN37" t="n">
         <v>4</v>
       </c>
-      <c r="AH37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI37" t="n">
-        <v>2</v>
-      </c>
-      <c r="AJ37" t="n">
-        <v>2</v>
-      </c>
-      <c r="AK37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM37" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN37" t="n">
-        <v>3</v>
-      </c>
       <c r="AO37" t="n">
         <v>0</v>
       </c>
       <c r="AP37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AQ37" t="n">
         <v>0</v>
@@ -9480,7 +9480,7 @@
         <v>1</v>
       </c>
       <c r="AU37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AV37" t="n">
         <v>1</v>
@@ -9489,7 +9489,7 @@
         <v>0</v>
       </c>
       <c r="AX37" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38">
@@ -9573,67 +9573,67 @@
         </is>
       </c>
       <c r="AD38" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="AE38" t="n">
+        <v>14</v>
+      </c>
+      <c r="AF38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG38" t="n">
         <v>11</v>
       </c>
-      <c r="AF38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG38" t="n">
+      <c r="AH38" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI38" t="n">
+        <v>3</v>
+      </c>
+      <c r="AJ38" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN38" t="n">
+        <v>5</v>
+      </c>
+      <c r="AO38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP38" t="n">
+        <v>4</v>
+      </c>
+      <c r="AQ38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT38" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU38" t="n">
+        <v>6</v>
+      </c>
+      <c r="AV38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX38" t="n">
         <v>9</v>
-      </c>
-      <c r="AH38" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI38" t="n">
-        <v>2</v>
-      </c>
-      <c r="AJ38" t="n">
-        <v>2</v>
-      </c>
-      <c r="AK38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM38" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN38" t="n">
-        <v>4</v>
-      </c>
-      <c r="AO38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP38" t="n">
-        <v>3</v>
-      </c>
-      <c r="AQ38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS38" t="n">
-        <v>1</v>
-      </c>
-      <c r="AT38" t="n">
-        <v>2</v>
-      </c>
-      <c r="AU38" t="n">
-        <v>5</v>
-      </c>
-      <c r="AV38" t="n">
-        <v>1</v>
-      </c>
-      <c r="AW38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX38" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="39">
@@ -9717,67 +9717,67 @@
         </is>
       </c>
       <c r="AD39" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="AE39" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="AF39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG39" t="n">
+        <v>12</v>
+      </c>
+      <c r="AH39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AI39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AJ39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AK39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN39" t="n">
+        <v>7</v>
+      </c>
+      <c r="AO39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP39" t="n">
+        <v>6</v>
+      </c>
+      <c r="AQ39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT39" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU39" t="n">
+        <v>9</v>
+      </c>
+      <c r="AV39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX39" t="n">
         <v>10</v>
-      </c>
-      <c r="AH39" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI39" t="n">
-        <v>3</v>
-      </c>
-      <c r="AJ39" t="n">
-        <v>3</v>
-      </c>
-      <c r="AK39" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL39" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM39" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN39" t="n">
-        <v>5</v>
-      </c>
-      <c r="AO39" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP39" t="n">
-        <v>4</v>
-      </c>
-      <c r="AQ39" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR39" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS39" t="n">
-        <v>1</v>
-      </c>
-      <c r="AT39" t="n">
-        <v>2</v>
-      </c>
-      <c r="AU39" t="n">
-        <v>7</v>
-      </c>
-      <c r="AV39" t="n">
-        <v>1</v>
-      </c>
-      <c r="AW39" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX39" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="40">
@@ -9861,26 +9861,26 @@
         </is>
       </c>
       <c r="AD40" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="AE40" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="AF40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG40" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AH40" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AI40" t="n">
+        <v>5</v>
+      </c>
+      <c r="AJ40" t="n">
         <v>4</v>
       </c>
-      <c r="AJ40" t="n">
-        <v>3</v>
-      </c>
       <c r="AK40" t="n">
         <v>0</v>
       </c>
@@ -9891,13 +9891,13 @@
         <v>1</v>
       </c>
       <c r="AN40" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AO40" t="n">
         <v>1</v>
       </c>
       <c r="AP40" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AQ40" t="n">
         <v>0</v>
@@ -9912,7 +9912,7 @@
         <v>2</v>
       </c>
       <c r="AU40" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AV40" t="n">
         <v>1</v>
@@ -9921,7 +9921,7 @@
         <v>0</v>
       </c>
       <c r="AX40" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41">
@@ -10005,25 +10005,25 @@
         </is>
       </c>
       <c r="AD41" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="AE41" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="AF41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG41" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="AH41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AI41" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AJ41" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AK41" t="n">
         <v>0</v>
@@ -10035,13 +10035,13 @@
         <v>2</v>
       </c>
       <c r="AN41" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AO41" t="n">
         <v>1</v>
       </c>
       <c r="AP41" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AQ41" t="n">
         <v>0</v>
@@ -10056,7 +10056,7 @@
         <v>2</v>
       </c>
       <c r="AU41" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AV41" t="n">
         <v>1</v>
@@ -10065,7 +10065,7 @@
         <v>0</v>
       </c>
       <c r="AX41" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="42">
@@ -10149,26 +10149,26 @@
         </is>
       </c>
       <c r="AD42" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="AE42" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="AF42" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AG42" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="AH42" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AI42" t="n">
+        <v>7</v>
+      </c>
+      <c r="AJ42" t="n">
         <v>5</v>
       </c>
-      <c r="AJ42" t="n">
-        <v>3</v>
-      </c>
       <c r="AK42" t="n">
         <v>0</v>
       </c>
@@ -10179,13 +10179,13 @@
         <v>2</v>
       </c>
       <c r="AN42" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AO42" t="n">
         <v>1</v>
       </c>
       <c r="AP42" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AQ42" t="n">
         <v>0</v>
@@ -10200,7 +10200,7 @@
         <v>2</v>
       </c>
       <c r="AU42" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AV42" t="n">
         <v>1</v>
@@ -10209,7 +10209,7 @@
         <v>0</v>
       </c>
       <c r="AX42" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="43">
@@ -10293,26 +10293,26 @@
         </is>
       </c>
       <c r="AD43" t="n">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="AE43" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="AF43" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AG43" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="AH43" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AI43" t="n">
+        <v>7</v>
+      </c>
+      <c r="AJ43" t="n">
         <v>5</v>
       </c>
-      <c r="AJ43" t="n">
-        <v>3</v>
-      </c>
       <c r="AK43" t="n">
         <v>0</v>
       </c>
@@ -10323,13 +10323,13 @@
         <v>2</v>
       </c>
       <c r="AN43" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AO43" t="n">
         <v>1</v>
       </c>
       <c r="AP43" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AQ43" t="n">
         <v>0</v>
@@ -10344,7 +10344,7 @@
         <v>2</v>
       </c>
       <c r="AU43" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AV43" t="n">
         <v>1</v>
@@ -10353,7 +10353,7 @@
         <v>0</v>
       </c>
       <c r="AX43" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="44">
@@ -10437,25 +10437,25 @@
         </is>
       </c>
       <c r="AD44" t="n">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="AE44" t="n">
+        <v>26</v>
+      </c>
+      <c r="AF44" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG44" t="n">
         <v>18</v>
       </c>
-      <c r="AF44" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG44" t="n">
-        <v>14</v>
-      </c>
       <c r="AH44" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AI44" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AJ44" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AK44" t="n">
         <v>0</v>
@@ -10467,13 +10467,13 @@
         <v>2</v>
       </c>
       <c r="AN44" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AO44" t="n">
         <v>1</v>
       </c>
       <c r="AP44" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AQ44" t="n">
         <v>0</v>
@@ -10488,7 +10488,7 @@
         <v>2</v>
       </c>
       <c r="AU44" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AV44" t="n">
         <v>1</v>
@@ -10497,7 +10497,7 @@
         <v>0</v>
       </c>
       <c r="AX44" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="45">
@@ -10581,67 +10581,67 @@
         </is>
       </c>
       <c r="AD45" t="n">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="AE45" t="n">
+        <v>28</v>
+      </c>
+      <c r="AF45" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG45" t="n">
+        <v>20</v>
+      </c>
+      <c r="AH45" t="n">
+        <v>6</v>
+      </c>
+      <c r="AI45" t="n">
+        <v>8</v>
+      </c>
+      <c r="AJ45" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM45" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN45" t="n">
+        <v>9</v>
+      </c>
+      <c r="AO45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP45" t="n">
+        <v>7</v>
+      </c>
+      <c r="AQ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT45" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU45" t="n">
+        <v>11</v>
+      </c>
+      <c r="AV45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX45" t="n">
         <v>19</v>
-      </c>
-      <c r="AF45" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG45" t="n">
-        <v>15</v>
-      </c>
-      <c r="AH45" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI45" t="n">
-        <v>5</v>
-      </c>
-      <c r="AJ45" t="n">
-        <v>4</v>
-      </c>
-      <c r="AK45" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL45" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM45" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN45" t="n">
-        <v>5</v>
-      </c>
-      <c r="AO45" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP45" t="n">
-        <v>4</v>
-      </c>
-      <c r="AQ45" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR45" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS45" t="n">
-        <v>1</v>
-      </c>
-      <c r="AT45" t="n">
-        <v>2</v>
-      </c>
-      <c r="AU45" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV45" t="n">
-        <v>1</v>
-      </c>
-      <c r="AW45" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX45" t="n">
-        <v>13</v>
       </c>
     </row>
     <row r="46">
@@ -10725,25 +10725,25 @@
         </is>
       </c>
       <c r="AD46" t="n">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="AE46" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="AF46" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AG46" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="AH46" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AI46" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AJ46" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AK46" t="n">
         <v>0</v>
@@ -10752,16 +10752,16 @@
         <v>0</v>
       </c>
       <c r="AM46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AN46" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AO46" t="n">
         <v>1</v>
       </c>
       <c r="AP46" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AQ46" t="n">
         <v>0</v>
@@ -10776,7 +10776,7 @@
         <v>2</v>
       </c>
       <c r="AU46" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="AV46" t="n">
         <v>1</v>
@@ -10785,7 +10785,7 @@
         <v>0</v>
       </c>
       <c r="AX46" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="47">
@@ -10869,25 +10869,25 @@
         </is>
       </c>
       <c r="AD47" t="n">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="AE47" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="AF47" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AG47" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="AH47" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AI47" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="AJ47" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AK47" t="n">
         <v>1</v>
@@ -10896,16 +10896,16 @@
         <v>0</v>
       </c>
       <c r="AM47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AN47" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="AO47" t="n">
         <v>1</v>
       </c>
       <c r="AP47" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AQ47" t="n">
         <v>0</v>
@@ -10920,7 +10920,7 @@
         <v>3</v>
       </c>
       <c r="AU47" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="AV47" t="n">
         <v>1</v>
@@ -10929,7 +10929,7 @@
         <v>0</v>
       </c>
       <c r="AX47" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="48">
@@ -11013,25 +11013,25 @@
         </is>
       </c>
       <c r="AD48" t="n">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="AE48" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="AF48" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AG48" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="AH48" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AI48" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="AJ48" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AK48" t="n">
         <v>1</v>
@@ -11040,16 +11040,16 @@
         <v>0</v>
       </c>
       <c r="AM48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AN48" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="AO48" t="n">
         <v>1</v>
       </c>
       <c r="AP48" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AQ48" t="n">
         <v>0</v>
@@ -11064,7 +11064,7 @@
         <v>3</v>
       </c>
       <c r="AU48" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="AV48" t="n">
         <v>1</v>
@@ -11073,7 +11073,7 @@
         <v>0</v>
       </c>
       <c r="AX48" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="49">
@@ -11157,43 +11157,43 @@
         </is>
       </c>
       <c r="AD49" t="n">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AE49" t="n">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="AF49" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AG49" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="AH49" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="AI49" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="AJ49" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="AK49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AL49" t="n">
         <v>0</v>
       </c>
       <c r="AM49" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AN49" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="AO49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AP49" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AQ49" t="n">
         <v>0</v>
@@ -11202,13 +11202,13 @@
         <v>1</v>
       </c>
       <c r="AS49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT49" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AU49" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="AV49" t="n">
         <v>1</v>
@@ -11217,7 +11217,7 @@
         <v>0</v>
       </c>
       <c r="AX49" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="50">
@@ -11301,43 +11301,43 @@
         </is>
       </c>
       <c r="AD50" t="n">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="AE50" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="AF50" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AG50" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="AH50" t="n">
+        <v>11</v>
+      </c>
+      <c r="AI50" t="n">
+        <v>11</v>
+      </c>
+      <c r="AJ50" t="n">
+        <v>13</v>
+      </c>
+      <c r="AK50" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM50" t="n">
         <v>4</v>
       </c>
-      <c r="AI50" t="n">
-        <v>7</v>
-      </c>
-      <c r="AJ50" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK50" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL50" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM50" t="n">
-        <v>3</v>
-      </c>
       <c r="AN50" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="AO50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AP50" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="AQ50" t="n">
         <v>0</v>
@@ -11346,13 +11346,13 @@
         <v>1</v>
       </c>
       <c r="AS50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AU50" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="AV50" t="n">
         <v>1</v>
@@ -11361,7 +11361,7 @@
         <v>0</v>
       </c>
       <c r="AX50" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
     </row>
     <row r="51">
@@ -11445,43 +11445,43 @@
         </is>
       </c>
       <c r="AD51" t="n">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="AE51" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="AF51" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AG51" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="AH51" t="n">
+        <v>11</v>
+      </c>
+      <c r="AI51" t="n">
+        <v>11</v>
+      </c>
+      <c r="AJ51" t="n">
+        <v>13</v>
+      </c>
+      <c r="AK51" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM51" t="n">
         <v>4</v>
       </c>
-      <c r="AI51" t="n">
-        <v>7</v>
-      </c>
-      <c r="AJ51" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK51" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL51" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM51" t="n">
-        <v>3</v>
-      </c>
       <c r="AN51" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="AO51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AP51" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="AQ51" t="n">
         <v>0</v>
@@ -11490,22 +11490,22 @@
         <v>1</v>
       </c>
       <c r="AS51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT51" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AU51" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="AV51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW51" t="n">
         <v>0</v>
       </c>
       <c r="AX51" t="n">
-        <v>17</v>
+        <v>28</v>
       </c>
     </row>
     <row r="52">
@@ -11589,67 +11589,67 @@
         </is>
       </c>
       <c r="AD52" t="n">
-        <v>82</v>
+        <v>110</v>
       </c>
       <c r="AE52" t="n">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="AF52" t="n">
+        <v>7</v>
+      </c>
+      <c r="AG52" t="n">
+        <v>35</v>
+      </c>
+      <c r="AH52" t="n">
+        <v>14</v>
+      </c>
+      <c r="AI52" t="n">
+        <v>14</v>
+      </c>
+      <c r="AJ52" t="n">
+        <v>15</v>
+      </c>
+      <c r="AK52" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM52" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN52" t="n">
+        <v>16</v>
+      </c>
+      <c r="AO52" t="n">
         <v>4</v>
       </c>
-      <c r="AG52" t="n">
-        <v>23</v>
-      </c>
-      <c r="AH52" t="n">
-        <v>5</v>
-      </c>
-      <c r="AI52" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ52" t="n">
-        <v>8</v>
-      </c>
-      <c r="AK52" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL52" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM52" t="n">
+      <c r="AP52" t="n">
+        <v>12</v>
+      </c>
+      <c r="AQ52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR52" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS52" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT52" t="n">
         <v>4</v>
       </c>
-      <c r="AN52" t="n">
-        <v>7</v>
-      </c>
-      <c r="AO52" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP52" t="n">
-        <v>6</v>
-      </c>
-      <c r="AQ52" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR52" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS52" t="n">
-        <v>1</v>
-      </c>
-      <c r="AT52" t="n">
-        <v>3</v>
-      </c>
       <c r="AU52" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="AV52" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX52" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
     </row>
     <row r="53">
@@ -11733,43 +11733,43 @@
         </is>
       </c>
       <c r="AD53" t="n">
-        <v>84</v>
+        <v>114</v>
       </c>
       <c r="AE53" t="n">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="AF53" t="n">
+        <v>7</v>
+      </c>
+      <c r="AG53" t="n">
+        <v>35</v>
+      </c>
+      <c r="AH53" t="n">
+        <v>14</v>
+      </c>
+      <c r="AI53" t="n">
+        <v>14</v>
+      </c>
+      <c r="AJ53" t="n">
+        <v>16</v>
+      </c>
+      <c r="AK53" t="n">
         <v>4</v>
       </c>
-      <c r="AG53" t="n">
-        <v>23</v>
-      </c>
-      <c r="AH53" t="n">
+      <c r="AL53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM53" t="n">
         <v>5</v>
       </c>
-      <c r="AI53" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ53" t="n">
-        <v>8</v>
-      </c>
-      <c r="AK53" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL53" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM53" t="n">
+      <c r="AN53" t="n">
+        <v>16</v>
+      </c>
+      <c r="AO53" t="n">
         <v>4</v>
       </c>
-      <c r="AN53" t="n">
-        <v>7</v>
-      </c>
-      <c r="AO53" t="n">
-        <v>2</v>
-      </c>
       <c r="AP53" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="AQ53" t="n">
         <v>0</v>
@@ -11778,22 +11778,22 @@
         <v>2</v>
       </c>
       <c r="AS53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT53" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AU53" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="AV53" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX53" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
     </row>
     <row r="54">
@@ -11877,43 +11877,43 @@
         </is>
       </c>
       <c r="AD54" t="n">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="AE54" t="n">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="AF54" t="n">
+        <v>7</v>
+      </c>
+      <c r="AG54" t="n">
+        <v>36</v>
+      </c>
+      <c r="AH54" t="n">
+        <v>14</v>
+      </c>
+      <c r="AI54" t="n">
+        <v>14</v>
+      </c>
+      <c r="AJ54" t="n">
+        <v>16</v>
+      </c>
+      <c r="AK54" t="n">
         <v>4</v>
       </c>
-      <c r="AG54" t="n">
-        <v>23</v>
-      </c>
-      <c r="AH54" t="n">
+      <c r="AL54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM54" t="n">
         <v>5</v>
       </c>
-      <c r="AI54" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ54" t="n">
-        <v>8</v>
-      </c>
-      <c r="AK54" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL54" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM54" t="n">
+      <c r="AN54" t="n">
+        <v>17</v>
+      </c>
+      <c r="AO54" t="n">
         <v>4</v>
       </c>
-      <c r="AN54" t="n">
-        <v>7</v>
-      </c>
-      <c r="AO54" t="n">
-        <v>2</v>
-      </c>
       <c r="AP54" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="AQ54" t="n">
         <v>0</v>
@@ -11922,22 +11922,22 @@
         <v>2</v>
       </c>
       <c r="AS54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT54" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AU54" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="AV54" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX54" t="n">
-        <v>18</v>
+        <v>34</v>
       </c>
     </row>
     <row r="55">
@@ -107750,13 +107750,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2AF050FD-5C69-46E0-A80C-4F72FE142D7A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75127CD3-F994-40A2-AF90-DA83A6640AB0}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48ED3200-3784-4603-AE93-3EA59C45CD5E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84C31AEB-A8C0-4A27-BF9C-F71FBC13F845}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{924E9511-49FA-43BA-B068-6DB09D661A55}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A2322465-516B-4BC3-9974-A5FB34374AA9}"/>
 </file>
</xml_diff>